<commit_message>
planilla UOCRA: desplegables de mes que funcionan en Google Sheets
La compradora no podía elegir el mes «Hasta» en la hoja Diferencias. exceljs le saca
los «$» a la lista de validación y junta las celdas con validación idéntica en un solo
rango (B8:B9): al importar, Google Sheets le corría una fila la lista a la segunda celda.

- Cada desplegable de mes lee una columna de su misma hoja (antes, la fila de
  encabezados de «Escalas») y lleva su propio mensaje, así no se fusiona.
- check_planilla_uocra_diferencias: ningún desplegable lee de otra hoja, «Desde» y
  «Hasta» no comparten regla, y los tres ofrecen los 30 meses.
- Verificado en un Google Sheet nativo convertido desde el archivo: los desplegables
  apuntan a Diferencias!A16:A45 y el total coincide con HyperFormula y con el cálculo a mano.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-uocra-2026.xlsx
+++ b/private/planilla-uocra-2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="229">
   <si>
     <t>Cómo usar esta planilla</t>
   </si>
@@ -5825,13 +5825,14 @@
   <sheetPr>
     <tabColor rgb="FF1B5E20"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="4" customWidth="1"/>
     <col min="4" max="5" width="18" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -5852,7 +5853,7 @@
       </c>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>25</v>
       </c>
@@ -5862,8 +5863,11 @@
       <c r="D5">
         <f>MATCH(B7,'Escalas'!$D$2:$AG$2,0)</f>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>26</v>
       </c>
@@ -5873,8 +5877,11 @@
       <c r="D6">
         <f>CONCATENATE("J|",B5,"|",B6)</f>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>113</v>
       </c>
@@ -5884,8 +5891,11 @@
       <c r="D7">
         <f>INDEX('Escalas'!$D$3:$AG$22,MATCH(D6,'Escalas'!$A$3:$A$22,0),D5)</f>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>114</v>
       </c>
@@ -5895,8 +5905,11 @@
       <c r="D8">
         <f>CONCATENATE("S|",B5,"|",B6)</f>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>115</v>
       </c>
@@ -5906,8 +5919,11 @@
       <c r="D9">
         <f>INDEX('Escalas'!$D$24:$AG$43,MATCH(D8,'Escalas'!$A$24:$A$43,0),D5)</f>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>117</v>
       </c>
@@ -5917,132 +5933,219 @@
       <c r="D10">
         <f>IF(B5="Sereno",1,0)</f>
       </c>
-    </row>
-    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" ht="6" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>118</v>
       </c>
       <c r="B12" s="4"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
         <v>119</v>
       </c>
       <c r="B13" s="22">
         <f>IF(D10=1,"—",D7)</f>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>120</v>
       </c>
       <c r="B14" s="23">
         <f>IF(D10=1,"—",B8)</f>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>121</v>
       </c>
       <c r="B15" s="22">
         <f>IF(D10=1,D7,D7*B8)</f>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B16" s="22">
         <f>IF(B9="Sí",B15*0.2,0)</f>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
         <v>123</v>
       </c>
       <c r="B17" s="22">
         <f>B15+B16</f>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
         <v>124</v>
       </c>
       <c r="B18" s="22">
         <f>D9</f>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>125</v>
       </c>
       <c r="B19" s="25">
         <f>B17+B18</f>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
         <v>126</v>
       </c>
       <c r="B20" s="22">
         <f>-(B17*(0.17+IF(B10="Sí",0.02,0))+B18*0.03)</f>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>127</v>
       </c>
       <c r="B21" s="25">
         <f>B19+B20</f>
       </c>
-    </row>
-    <row r="22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" ht="6" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>128</v>
       </c>
       <c r="B23" s="4"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>129</v>
       </c>
       <c r="B24" s="22">
         <f>B17*0.12</f>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
         <v>130</v>
       </c>
       <c r="B25" s="22">
         <f>B17*0.08</f>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>131</v>
       </c>
       <c r="B27" s="6"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>132</v>
       </c>
       <c r="B28" s="6"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>133</v>
       </c>
       <c r="B29" s="6"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>134</v>
       </c>
       <c r="B30" s="6"/>
+      <c r="G30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -6067,7 +6170,7 @@
       <formula1>"Zona A,Zona B,Zona C,Zona C Austral"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B7">
-      <formula1>'Escalas'!$D$2:$AG$2</formula1>
+      <formula1>'Liquidador'!G5:G34</formula1>
     </dataValidation>
     <dataValidation type="decimal" showErrorMessage="1" error="Ingresá las horas del mes (entre 1 y 300). Mes completo = 190,67." sqref="B8">
       <formula1>1</formula1>
@@ -8037,7 +8140,7 @@
     <mergeCell ref="A60:K60"/>
     <mergeCell ref="A61:K61"/>
   </mergeCells>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="list" showErrorMessage="1" error="Elegí Sí o No." sqref="B10">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
@@ -8058,8 +8161,11 @@
     <dataValidation type="list" showErrorMessage="1" error="Elegí una zona." sqref="B7">
       <formula1>"Zona A,Zona B,Zona C,Zona C Austral"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B8:B9">
-      <formula1>'Escalas'!$D$2:$AG$2</formula1>
+    <dataValidation type="list" showErrorMessage="1" error="Elegí el primer mes del reclamo." sqref="B8">
+      <formula1>'Diferencias'!A16:A45</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" error="Elegí el último mes del reclamo." sqref="B9">
+      <formula1>'Diferencias'!A16:A45</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
planilla UOCRA: desplegables de mes que funcionan en Google Sheets (#54)
La compradora no podía elegir el mes «Hasta» en la hoja Diferencias. exceljs le saca
los «$» a la lista de validación y junta las celdas con validación idéntica en un solo
rango (B8:B9): al importar, Google Sheets le corría una fila la lista a la segunda celda.

- Cada desplegable de mes lee una columna de su misma hoja (antes, la fila de
  encabezados de «Escalas») y lleva su propio mensaje, así no se fusiona.
- check_planilla_uocra_diferencias: ningún desplegable lee de otra hoja, «Desde» y
  «Hasta» no comparten regla, y los tres ofrecen los 30 meses.
- Verificado en un Google Sheet nativo convertido desde el archivo: los desplegables
  apuntan a Diferencias!A16:A45 y el total coincide con HyperFormula y con el cálculo a mano.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-uocra-2026.xlsx
+++ b/private/planilla-uocra-2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="229">
   <si>
     <t>Cómo usar esta planilla</t>
   </si>
@@ -5825,13 +5825,14 @@
   <sheetPr>
     <tabColor rgb="FF1B5E20"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="4" customWidth="1"/>
     <col min="4" max="5" width="18" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -5852,7 +5853,7 @@
       </c>
       <c r="B4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>25</v>
       </c>
@@ -5862,8 +5863,11 @@
       <c r="D5">
         <f>MATCH(B7,'Escalas'!$D$2:$AG$2,0)</f>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>26</v>
       </c>
@@ -5873,8 +5877,11 @@
       <c r="D6">
         <f>CONCATENATE("J|",B5,"|",B6)</f>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
         <v>113</v>
       </c>
@@ -5884,8 +5891,11 @@
       <c r="D7">
         <f>INDEX('Escalas'!$D$3:$AG$22,MATCH(D6,'Escalas'!$A$3:$A$22,0),D5)</f>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
         <v>114</v>
       </c>
@@ -5895,8 +5905,11 @@
       <c r="D8">
         <f>CONCATENATE("S|",B5,"|",B6)</f>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
         <v>115</v>
       </c>
@@ -5906,8 +5919,11 @@
       <c r="D9">
         <f>INDEX('Escalas'!$D$24:$AG$43,MATCH(D8,'Escalas'!$A$24:$A$43,0),D5)</f>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
         <v>117</v>
       </c>
@@ -5917,132 +5933,219 @@
       <c r="D10">
         <f>IF(B5="Sereno",1,0)</f>
       </c>
-    </row>
-    <row r="11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" ht="6" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>118</v>
       </c>
       <c r="B12" s="4"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
         <v>119</v>
       </c>
       <c r="B13" s="22">
         <f>IF(D10=1,"—",D7)</f>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>120</v>
       </c>
       <c r="B14" s="23">
         <f>IF(D10=1,"—",B8)</f>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>121</v>
       </c>
       <c r="B15" s="22">
         <f>IF(D10=1,D7,D7*B8)</f>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
         <v>122</v>
       </c>
       <c r="B16" s="22">
         <f>IF(B9="Sí",B15*0.2,0)</f>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
         <v>123</v>
       </c>
       <c r="B17" s="22">
         <f>B15+B16</f>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
         <v>124</v>
       </c>
       <c r="B18" s="22">
         <f>D9</f>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>125</v>
       </c>
       <c r="B19" s="25">
         <f>B17+B18</f>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
         <v>126</v>
       </c>
       <c r="B20" s="22">
         <f>-(B17*(0.17+IF(B10="Sí",0.02,0))+B18*0.03)</f>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>127</v>
       </c>
       <c r="B21" s="25">
         <f>B19+B20</f>
       </c>
-    </row>
-    <row r="22" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" ht="6" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>128</v>
       </c>
       <c r="B23" s="4"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
         <v>129</v>
       </c>
       <c r="B24" s="22">
         <f>B17*0.12</f>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
         <v>130</v>
       </c>
       <c r="B25" s="22">
         <f>B17*0.08</f>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G25" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>131</v>
       </c>
       <c r="B27" s="6"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G27" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>132</v>
       </c>
       <c r="B28" s="6"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G28" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>133</v>
       </c>
       <c r="B29" s="6"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>134</v>
       </c>
       <c r="B30" s="6"/>
+      <c r="G30" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G34" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -6067,7 +6170,7 @@
       <formula1>"Zona A,Zona B,Zona C,Zona C Austral"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B7">
-      <formula1>'Escalas'!$D$2:$AG$2</formula1>
+      <formula1>'Liquidador'!G5:G34</formula1>
     </dataValidation>
     <dataValidation type="decimal" showErrorMessage="1" error="Ingresá las horas del mes (entre 1 y 300). Mes completo = 190,67." sqref="B8">
       <formula1>1</formula1>
@@ -8037,7 +8140,7 @@
     <mergeCell ref="A60:K60"/>
     <mergeCell ref="A61:K61"/>
   </mergeCells>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation type="list" showErrorMessage="1" error="Elegí Sí o No." sqref="B10">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
@@ -8058,8 +8161,11 @@
     <dataValidation type="list" showErrorMessage="1" error="Elegí una zona." sqref="B7">
       <formula1>"Zona A,Zona B,Zona C,Zona C Austral"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B8:B9">
-      <formula1>'Escalas'!$D$2:$AG$2</formula1>
+    <dataValidation type="list" showErrorMessage="1" error="Elegí el primer mes del reclamo." sqref="B8">
+      <formula1>'Diferencias'!A16:A45</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" error="Elegí el último mes del reclamo." sqref="B9">
+      <formula1>'Diferencias'!A16:A45</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>